<commit_message>
Inserito Import Chiavi, inseritarichiesta ferie permessi, parametrizzato utilizzo inizio giornata, inserito import note dalle app, modificato import excel dei cantieri, inserito campo raggio, ripristinato funzionamento filiali e responsabili
</commit_message>
<xml_diff>
--- a/PowerWeb/ExcelModels/Cdc.xlsx
+++ b/PowerWeb/ExcelModels/Cdc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\backup\PWNuovo\PowerWeb\ExcelModels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D4AC9A3-370F-43A1-AB08-D744DE5DF629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE0694F-384A-409E-93B6-0EA8279D5200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="990" yWindow="-120" windowWidth="27930" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -103,8 +103,6 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -115,6 +113,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -397,29 +401,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A2:M2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39" style="3" customWidth="1"/>
-    <col min="2" max="2" width="41.42578125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="1"/>
-    <col min="6" max="6" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" style="1"/>
+    <col min="1" max="1" width="39" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="2"/>
+    <col min="6" max="6" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="2"/>
+    <col min="8" max="11" width="9.140625" style="6"/>
+    <col min="12" max="13" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>